<commit_message>
Add support for NULL values
</commit_message>
<xml_diff>
--- a/src/test/resources/teda/xlsx/DIFFERENT_DATABASE_TEST.xlsx
+++ b/src/test/resources/teda/xlsx/DIFFERENT_DATABASE_TEST.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pad\Projects\teda\src\test\resources\teda\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\teda-framework\src\test\resources\teda\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2114AE66-5F4F-45D5-93CE-14F79B9A6096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13784ECF-302A-4E22-AFDD-847DBAAA2743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="1140" windowWidth="19200" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="51420" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cockpit" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="23">
   <si>
     <t>#Teda</t>
   </si>
@@ -88,9 +88,6 @@
   </si>
   <si>
     <t>#ID</t>
-  </si>
-  <si>
-    <t>FOO_BAR</t>
   </si>
   <si>
     <t>DifferentDatabaseTest</t>
@@ -199,8 +196,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table13578" displayName="Table13578" ref="C4:F8" totalsRowShown="0">
   <autoFilter ref="C4:F8" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="ID" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="NAME" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="ID" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="NAME" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="AGE"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="AVERAGE"/>
   </tableColumns>
@@ -209,22 +206,22 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table4" displayName="Table4" ref="C4:F5" insertRow="1">
-  <autoFilter ref="C4:F5" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table4" displayName="Table4" ref="C4:F8">
+  <autoFilter ref="C4:F8" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="#ID" totalsRowLabel="Ergebnis" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="NAME" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="#ID" totalsRowLabel="Ergebnis" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="NAME" dataDxfId="0"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="AGE"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="AVERAGE" totalsRowFunction="sum" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="AVERAGE" totalsRowFunction="sum" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -262,9 +259,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -297,26 +294,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -349,26 +329,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -557,7 +520,7 @@
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.35">
@@ -582,7 +545,7 @@
         <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F5" t="s">
         <v>12</v>
@@ -796,24 +759,60 @@
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="F5" s="2"/>
+      <c r="C5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5">
+        <v>22</v>
+      </c>
+      <c r="F5">
+        <v>12.66</v>
+      </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="F6" s="2"/>
+      <c r="C6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6">
+        <v>45</v>
+      </c>
+      <c r="F6">
+        <v>34.44</v>
+      </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="F7" s="2"/>
+      <c r="C7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7">
+        <v>21</v>
+      </c>
+      <c r="F7">
+        <v>24.33</v>
+      </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="F8" s="4"/>
+      <c r="C8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8">
+        <v>66</v>
+      </c>
+      <c r="F8" s="4">
+        <v>4.3939494940000001</v>
+      </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.35">
       <c r="C9" s="2"/>

</xml_diff>